<commit_message>
Update formatting in deployment summary template
</commit_message>
<xml_diff>
--- a/log_templates/OBS_Deployment_Summary_Template.xlsx
+++ b/log_templates/OBS_Deployment_Summary_Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Katie Bosman\code\OBSDataPipeline\log_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B7A4C26-23EF-402C-B993-F69B99E2C167}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1AE1E84-6086-45CA-BD79-CEA707DBA3E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-10910" windowWidth="38620" windowHeight="21220" xr2:uid="{40123D5C-8A56-48C8-83AB-25C6150FC8B9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{40123D5C-8A56-48C8-83AB-25C6150FC8B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Locations" sheetId="1" r:id="rId1"/>
@@ -217,7 +217,7 @@
     <numFmt numFmtId="164" formatCode="yyyy/mm/dd\ hh:mm:ss"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -233,16 +233,41 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -259,14 +284,29 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -288,8 +328,28 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="2" xfId="2" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
+    <cellStyle name="Calculation" xfId="2" builtinId="22"/>
+    <cellStyle name="Input" xfId="1" builtinId="20"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -605,242 +665,309 @@
   <dimension ref="A1:AE14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="11.5703125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="26.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.85546875" customWidth="1"/>
-    <col min="20" max="20" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.28515625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="8"/>
+    <col min="3" max="3" width="9.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="9" width="18.28515625" style="9" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.140625" style="8"/>
+    <col min="11" max="11" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.140625" style="8"/>
+    <col min="14" max="14" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10" style="8" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="26.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.140625" style="11"/>
+    <col min="18" max="18" width="9.85546875" style="11" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.85546875" style="11" customWidth="1"/>
+    <col min="20" max="20" width="11.140625" style="11" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.28515625" style="11" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.85546875" style="11" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="9.140625" style="8"/>
+    <col min="30" max="30" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="26.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="32" max="16384" width="9.140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
+    <row r="1" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="6"/>
-      <c r="D1" s="7" t="s">
+      <c r="C1" s="4"/>
+      <c r="D1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="6" t="s">
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
-      <c r="M1" s="6" t="s">
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="N1" s="6"/>
-      <c r="O1" s="6"/>
-      <c r="P1" s="6"/>
-      <c r="Q1" s="6" t="s">
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="R1" s="6"/>
-      <c r="S1" s="6"/>
-      <c r="T1" s="6"/>
-      <c r="U1" s="6"/>
-      <c r="V1" s="6"/>
-      <c r="W1" s="6"/>
-      <c r="X1" s="6"/>
-      <c r="Y1" s="6" t="s">
+      <c r="R1" s="4"/>
+      <c r="S1" s="4"/>
+      <c r="T1" s="4"/>
+      <c r="U1" s="4"/>
+      <c r="V1" s="4"/>
+      <c r="W1" s="4"/>
+      <c r="X1" s="4"/>
+      <c r="Y1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="6"/>
-      <c r="AA1" s="6"/>
-      <c r="AB1" s="6"/>
-      <c r="AC1" s="6" t="s">
+      <c r="Z1" s="4"/>
+      <c r="AA1" s="4"/>
+      <c r="AB1" s="4"/>
+      <c r="AC1" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="AD1" s="6"/>
-      <c r="AE1" s="6"/>
-    </row>
-    <row r="2" spans="1:31" s="4" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="4" t="s">
+      <c r="AD1" s="4"/>
+      <c r="AE1" s="4"/>
+    </row>
+    <row r="2" spans="1:31" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="P2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="Q2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="R2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="S2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="T2" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="U2" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="V2" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="W2" s="4" t="s">
+      <c r="W2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="X2" s="4" t="s">
+      <c r="X2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="Y2" s="4" t="s">
+      <c r="Y2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="Z2" s="4" t="s">
+      <c r="Z2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="AA2" s="4" t="s">
+      <c r="AA2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="AB2" s="4" t="s">
+      <c r="AB2" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="AC2" s="4" t="s">
+      <c r="AC2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="AD2" s="4" t="s">
+      <c r="AD2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="AE2" s="4" t="s">
+      <c r="AE2" s="2" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P3" s="2">
-        <f t="shared" ref="P3" si="0">2*6370*ASIN(SQRT(SIN(RADIANS(M3-J3)/2)*SIN(RADIANS(M3-J3)/2) + COS(RADIANS(M3))*COS(RADIANS(J3))*SIN(RADIANS(N3-K3)/2)*SIN(RADIANS(N3-K3)/2)))</f>
-        <v>0</v>
-      </c>
-      <c r="W3" s="2">
-        <f>2*6370*ASIN(SQRT(SIN(RADIANS(Q3-M3)/2)*SIN(RADIANS(Q3-M3)/2) + COS(RADIANS(Q3))*COS(RADIANS(M3))*SIN(RADIANS(R3-N3)/2)*SIN(RADIANS(R3-N3)/2)))*1000</f>
-        <v>0</v>
-      </c>
-      <c r="X3" t="e">
-        <f>MOD(DEGREES(ATAN2(COS(RADIANS(M3))*SIN(RADIANS(Q3)) - SIN(RADIANS(M3))*COS(RADIANS(Q3))*COS(RADIANS(R3-N3)),COS(RADIANS(Q3))*SIN(RADIANS(R3-N3)))) + 360, 360)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="AA3" s="2">
-        <f>2*6370*ASIN(SQRT(SIN(RADIANS(Y3-Q3)/2)*SIN(RADIANS(Y3-Q3)/2) + COS(RADIANS(Y3))*COS(RADIANS(Q3))*SIN(RADIANS(Z3-R3)/2)*SIN(RADIANS(Z3-R3)/2)))*1000</f>
-        <v>0</v>
-      </c>
-      <c r="AB3" t="e">
-        <f>MOD(DEGREES(ATAN2(COS(RADIANS(Q3))*SIN(RADIANS(Y3)) - SIN(RADIANS(Q3))*COS(RADIANS(Y3))*COS(RADIANS(Z3-R3)),COS(RADIANS(Y3))*SIN(RADIANS(Z3-R3)))) + 360, 360)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="AE3" s="2">
-        <f>2*6370*ASIN(SQRT(SIN(RADIANS(AC3-Y3)/2)*SIN(RADIANS(AC3-Y3)/2) + COS(RADIANS(AC3))*COS(RADIANS(Y3))*SIN(RADIANS(AD3-AA3)/2)*SIN(RADIANS(AD3-AA3)/2)))</f>
-        <v>0</v>
+      <c r="A3" s="8">
+        <f>'Deployment Log'!A3</f>
+        <v>0</v>
+      </c>
+      <c r="B3" s="8">
+        <f>'Deployment Log'!N3</f>
+        <v>0</v>
+      </c>
+      <c r="C3" s="8">
+        <f>'Deployment Log'!O3</f>
+        <v>0</v>
+      </c>
+      <c r="D3" s="9">
+        <f>'Deployment Log'!I3</f>
+        <v>0</v>
+      </c>
+      <c r="E3" s="9">
+        <f>'Deployment Log'!J3</f>
+        <v>0</v>
+      </c>
+      <c r="F3" s="9">
+        <f>'Deployment Log'!K3</f>
+        <v>0</v>
+      </c>
+      <c r="G3" s="9">
+        <f>'Recovery Log'!J3</f>
+        <v>0</v>
+      </c>
+      <c r="H3" s="9">
+        <f>'Recovery Log'!K3</f>
+        <v>0</v>
+      </c>
+      <c r="I3" s="9">
+        <f>'Recovery Log'!L3</f>
+        <v>0</v>
+      </c>
+      <c r="J3" s="8">
+        <f>'Deployment Log'!B3</f>
+        <v>0</v>
+      </c>
+      <c r="K3" s="8">
+        <f>'Deployment Log'!C3</f>
+        <v>0</v>
+      </c>
+      <c r="L3" s="8">
+        <f>'Deployment Log'!D3</f>
+        <v>0</v>
+      </c>
+      <c r="M3" s="8">
+        <f>'Deployment Log'!E3</f>
+        <v>0</v>
+      </c>
+      <c r="N3" s="8">
+        <f>'Deployment Log'!F3</f>
+        <v>0</v>
+      </c>
+      <c r="O3" s="8">
+        <f>'Deployment Log'!G3</f>
+        <v>0</v>
+      </c>
+      <c r="P3" s="10" t="str">
+        <f>'Deployment Log'!H3</f>
+        <v/>
+      </c>
+      <c r="W3" s="12" t="str">
+        <f>IF(ISBLANK(Q3),"",2*6370*ASIN(SQRT(SIN(RADIANS(Q3-M3)/2)*SIN(RADIANS(Q3-M3)/2) + COS(RADIANS(Q3))*COS(RADIANS(M3))*SIN(RADIANS(R3-N3)/2)*SIN(RADIANS(R3-N3)/2)))*1000)</f>
+        <v/>
+      </c>
+      <c r="X3" s="13" t="str">
+        <f>IF(ISBLANK(Q3),"",MOD(DEGREES(ATAN2(COS(RADIANS(M3))*SIN(RADIANS(Q3)) - SIN(RADIANS(M3))*COS(RADIANS(Q3))*COS(RADIANS(R3-N3)),COS(RADIANS(Q3))*SIN(RADIANS(R3-N3)))) + 360, 360))</f>
+        <v/>
+      </c>
+      <c r="Y3" s="8">
+        <f>'Recovery Log'!N3</f>
+        <v>0</v>
+      </c>
+      <c r="Z3" s="8">
+        <f>'Recovery Log'!O3</f>
+        <v>0</v>
+      </c>
+      <c r="AA3" s="10" t="str">
+        <f>'Recovery Log'!P3</f>
+        <v/>
+      </c>
+      <c r="AB3" s="13" t="str">
+        <f>IF(ISBLANK(Q3),"",MOD(DEGREES(ATAN2(COS(RADIANS(Q3))*SIN(RADIANS(Y3)) - SIN(RADIANS(Q3))*COS(RADIANS(Y3))*COS(RADIANS(Z3-R3)),COS(RADIANS(Y3))*SIN(RADIANS(Z3-R3)))) + 360, 360))</f>
+        <v/>
+      </c>
+      <c r="AC3" s="8">
+        <f>'Recovery Log'!Q3</f>
+        <v>0</v>
+      </c>
+      <c r="AD3" s="8">
+        <f>'Recovery Log'!R3</f>
+        <v>0</v>
+      </c>
+      <c r="AE3" s="10" t="str">
+        <f>'Recovery Log'!S3</f>
+        <v/>
       </c>
     </row>
     <row r="4" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P4" s="2"/>
-      <c r="W4" s="2"/>
+      <c r="P4" s="10"/>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P5" s="2"/>
-      <c r="W5" s="2"/>
+      <c r="P5" s="10"/>
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P6" s="2"/>
-      <c r="W6" s="2"/>
+      <c r="P6" s="10"/>
     </row>
     <row r="7" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P7" s="2"/>
-      <c r="W7" s="2"/>
+      <c r="P7" s="10"/>
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P8" s="2"/>
-      <c r="W8" s="2"/>
+      <c r="P8" s="10"/>
     </row>
     <row r="9" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P9" s="2"/>
-      <c r="W9" s="2"/>
+      <c r="P9" s="10"/>
     </row>
     <row r="10" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P10" s="2"/>
-      <c r="W10" s="2"/>
+      <c r="P10" s="10"/>
     </row>
     <row r="11" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P11" s="2"/>
-      <c r="W11" s="2"/>
+      <c r="P11" s="10"/>
     </row>
     <row r="12" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P12" s="2"/>
-      <c r="W12" s="2"/>
+      <c r="P12" s="10"/>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P13" s="2"/>
-      <c r="W13" s="2"/>
+      <c r="P13" s="10"/>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P14" s="2"/>
-      <c r="W14" s="2"/>
+      <c r="P14" s="10"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -910,253 +1037,259 @@
   <dimension ref="A1:AA14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.140625" customWidth="1"/>
-    <col min="10" max="10" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="10" customWidth="1"/>
-    <col min="20" max="20" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="20" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11" customWidth="1"/>
-    <col min="25" max="26" width="10.42578125" customWidth="1"/>
-    <col min="27" max="27" width="98.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="8"/>
+    <col min="3" max="3" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="8"/>
+    <col min="6" max="6" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" style="8" customWidth="1"/>
+    <col min="10" max="10" width="11.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.140625" style="8"/>
+    <col min="15" max="15" width="10" style="8" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="10" style="8" customWidth="1"/>
+    <col min="18" max="19" width="9.140625" style="8"/>
+    <col min="20" max="20" width="10.5703125" style="8" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.140625" style="8"/>
+    <col min="22" max="22" width="20" style="8" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11" style="8" customWidth="1"/>
+    <col min="25" max="26" width="10.42578125" style="8" customWidth="1"/>
+    <col min="27" max="27" width="98.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="28" max="16384" width="9.140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
+    <row r="1" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6" t="s">
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
-      <c r="I1" s="7" t="s">
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="6" t="s">
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="O1" s="6"/>
-      <c r="P1" s="6" t="s">
+      <c r="O1" s="4"/>
+      <c r="P1" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="Q1" s="6"/>
-      <c r="R1" s="6" t="s">
+      <c r="Q1" s="4"/>
+      <c r="R1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="S1" s="6"/>
-      <c r="T1" s="6" t="s">
+      <c r="S1" s="4"/>
+      <c r="T1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="U1" s="6"/>
-      <c r="V1" s="6"/>
-      <c r="W1" s="3" t="s">
+      <c r="U1" s="4"/>
+      <c r="V1" s="4"/>
+      <c r="W1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="X1" s="8" t="s">
+      <c r="X1" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="Y1" s="6" t="s">
+      <c r="Y1" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="Z1" s="6"/>
-      <c r="AA1" s="3" t="s">
+      <c r="Z1" s="4"/>
+      <c r="AA1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:27" s="4" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="4" t="s">
+    <row r="2" spans="1:27" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="J2" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="K2" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="L2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="M2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="P2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="Q2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="R2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="S2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="T2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="U2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="V2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="W2" s="4" t="s">
+      <c r="W2" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="X2" s="9"/>
-      <c r="Y2" s="4" t="s">
+      <c r="X2" s="7"/>
+      <c r="Y2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="Z2" s="4" t="s">
+      <c r="Z2" s="2" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H3" s="2">
-        <f t="shared" ref="H3" si="0">2*6370*ASIN(SQRT(SIN(RADIANS(E3-B3)/2)*SIN(RADIANS(E3-B3)/2) + COS(RADIANS(E3))*COS(RADIANS(B3))*SIN(RADIANS(F3-C3)/2)*SIN(RADIANS(F3-C3)/2)))</f>
-        <v>0</v>
-      </c>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
+      <c r="H3" s="12" t="str">
+        <f>IF(OR(ISBLANK(B3),ISBLANK(E3)),"",2*6370*ASIN(SQRT(SIN(RADIANS(E3-B3)/2)*SIN(RADIANS(E3-B3)/2) + COS(RADIANS(E3))*COS(RADIANS(B3))*SIN(RADIANS(F3-C3)/2)*SIN(RADIANS(F3-C3)/2))))</f>
+        <v/>
+      </c>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H4" s="2"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
+      <c r="H4" s="10"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H5" s="2"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H6" s="2"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H7" s="2"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H8" s="2"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H9" s="2"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
-      <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="9"/>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H10" s="2"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="1"/>
-      <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+      <c r="L10" s="9"/>
+      <c r="M10" s="9"/>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H11" s="2"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-      <c r="K11" s="1"/>
-      <c r="L11" s="1"/>
-      <c r="M11" s="1"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="9"/>
+      <c r="M11" s="9"/>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H12" s="2"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
-      <c r="L12" s="1"/>
-      <c r="M12" s="1"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="9"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="9"/>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H13" s="2"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="9"/>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H14" s="2"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -1192,145 +1325,169 @@
   <dimension ref="A1:X3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.42578125" customWidth="1"/>
-    <col min="11" max="12" width="9.140625" customWidth="1"/>
-    <col min="13" max="13" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.140625" customWidth="1"/>
-    <col min="15" max="15" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.140625" customWidth="1"/>
-    <col min="18" max="18" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="100.5703125" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="8"/>
+    <col min="3" max="3" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="8" width="9.140625" style="8"/>
+    <col min="9" max="9" width="15.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.42578125" style="8" customWidth="1"/>
+    <col min="11" max="12" width="9.140625" style="8" customWidth="1"/>
+    <col min="13" max="13" width="17.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.140625" style="8" customWidth="1"/>
+    <col min="15" max="15" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.140625" style="8" customWidth="1"/>
+    <col min="18" max="18" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="9.140625" style="8"/>
+    <col min="22" max="22" width="11.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="20.140625" style="8" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="100.5703125" style="8" customWidth="1"/>
+    <col min="25" max="16384" width="9.140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="3" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="6" t="s">
+    <row r="1" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6" t="s">
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6" t="s">
+      <c r="F1" s="4"/>
+      <c r="G1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="6"/>
-      <c r="I1" s="6" t="s">
+      <c r="H1" s="4"/>
+      <c r="I1" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="J1" s="6"/>
-      <c r="K1" s="6"/>
-      <c r="L1" s="6"/>
-      <c r="M1" s="6"/>
-      <c r="N1" s="6" t="s">
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="O1" s="6"/>
-      <c r="P1" s="6"/>
-      <c r="Q1" s="6" t="s">
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="R1" s="6"/>
-      <c r="S1" s="6"/>
-      <c r="T1" s="6" t="s">
+      <c r="R1" s="4"/>
+      <c r="S1" s="4"/>
+      <c r="T1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="U1" s="6"/>
-      <c r="V1" s="3" t="s">
+      <c r="U1" s="4"/>
+      <c r="V1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="W1" s="3" t="s">
+      <c r="W1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="X1" s="3" t="s">
+      <c r="X1" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:24" s="4" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="4" t="s">
+    <row r="2" spans="1:24" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="J2" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="L2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="N2" s="4" t="s">
+      <c r="N2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="O2" s="4" t="s">
+      <c r="O2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="P2" s="4" t="s">
+      <c r="P2" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="Q2" s="4" t="s">
+      <c r="Q2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="R2" s="4" t="s">
+      <c r="R2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="S2" s="4" t="s">
+      <c r="S2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="T2" s="4" t="s">
+      <c r="T2" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="U2" s="4" t="s">
+      <c r="U2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="V2" s="4" t="s">
+      <c r="V2" s="2" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="P3" s="2">
-        <f>2*6370*ASIN(SQRT(SIN(RADIANS(N3-B3)/2)*SIN(RADIANS(N3-B3)/2) + COS(RADIANS(N3))*COS(RADIANS(B3))*SIN(RADIANS(O3-C3)/2)*SIN(RADIANS(O3-C3)/2)))</f>
-        <v>0</v>
-      </c>
-      <c r="S3" s="2">
-        <f>2*6370*ASIN(SQRT(SIN(RADIANS(Q3-N3)/2)*SIN(RADIANS(Q3-N3)/2) + COS(RADIANS(Q3))*COS(RADIANS(N3))*SIN(RADIANS(R3-O3)/2)*SIN(RADIANS(R3-O3)/2)))</f>
-        <v>0</v>
+      <c r="A3" s="8">
+        <f>'Deployment Log'!A3</f>
+        <v>0</v>
+      </c>
+      <c r="E3" s="8">
+        <f>'Deployment Log'!N3</f>
+        <v>0</v>
+      </c>
+      <c r="F3" s="8">
+        <f>'Deployment Log'!O3</f>
+        <v>0</v>
+      </c>
+      <c r="G3" s="8">
+        <f>'Deployment Log'!R3</f>
+        <v>0</v>
+      </c>
+      <c r="H3" s="8">
+        <f>'Deployment Log'!S3</f>
+        <v>0</v>
+      </c>
+      <c r="P3" s="12" t="str">
+        <f>IF(ISBLANK(N3),"",2*6370*ASIN(SQRT(SIN(RADIANS(N3-B3)/2)*SIN(RADIANS(N3-B3)/2) + COS(RADIANS(N3))*COS(RADIANS(B3))*SIN(RADIANS(O3-C3)/2)*SIN(RADIANS(O3-C3)/2))))</f>
+        <v/>
+      </c>
+      <c r="S3" s="12" t="str">
+        <f>IF(OR(ISBLANK(N3),ISBLANK(Q3)),"",2*6370*ASIN(SQRT(SIN(RADIANS(Q3-N3)/2)*SIN(RADIANS(Q3-N3)/2) + COS(RADIANS(Q3))*COS(RADIANS(N3))*SIN(RADIANS(R3-O3)/2)*SIN(RADIANS(R3-O3)/2))))</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Small change to log template
</commit_message>
<xml_diff>
--- a/log_templates/OBS_Deployment_Summary_Template.xlsx
+++ b/log_templates/OBS_Deployment_Summary_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Katie Bosman\code\OBSDataPipeline\log_templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1AE1E84-6086-45CA-BD79-CEA707DBA3E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80D94346-8BDA-47C2-8638-E12A3FC13EC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{40123D5C-8A56-48C8-83AB-25C6150FC8B9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{40123D5C-8A56-48C8-83AB-25C6150FC8B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Locations" sheetId="1" r:id="rId1"/>
@@ -316,18 +316,6 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -345,6 +333,18 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="2" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -665,82 +665,82 @@
   <dimension ref="A1:AE14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="8"/>
-    <col min="3" max="3" width="9.7109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="9" width="18.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9.140625" style="8"/>
-    <col min="11" max="11" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.140625" style="8"/>
-    <col min="14" max="14" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10" style="8" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="26.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.140625" style="11"/>
-    <col min="18" max="18" width="9.85546875" style="11" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.85546875" style="11" customWidth="1"/>
-    <col min="20" max="20" width="11.140625" style="11" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.28515625" style="11" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.85546875" style="11" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="4"/>
+    <col min="3" max="3" width="9.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="9" width="18.28515625" style="5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.140625" style="4"/>
+    <col min="11" max="11" width="9.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.140625" style="4"/>
+    <col min="14" max="14" width="9.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="26.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.140625" style="7"/>
+    <col min="18" max="18" width="9.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.85546875" style="7" customWidth="1"/>
+    <col min="20" max="20" width="11.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.28515625" style="7" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.85546875" style="7" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="9.140625" style="8"/>
-    <col min="30" max="30" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="26.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="32" max="16384" width="9.140625" style="8"/>
+    <col min="29" max="29" width="9.140625" style="4"/>
+    <col min="30" max="30" width="9.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="26.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="32" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="5" t="s">
+      <c r="C1" s="10"/>
+      <c r="D1" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="4" t="s">
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4" t="s">
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4" t="s">
+      <c r="N1" s="10"/>
+      <c r="O1" s="10"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="R1" s="4"/>
-      <c r="S1" s="4"/>
-      <c r="T1" s="4"/>
-      <c r="U1" s="4"/>
-      <c r="V1" s="4"/>
-      <c r="W1" s="4"/>
-      <c r="X1" s="4"/>
-      <c r="Y1" s="4" t="s">
+      <c r="R1" s="10"/>
+      <c r="S1" s="10"/>
+      <c r="T1" s="10"/>
+      <c r="U1" s="10"/>
+      <c r="V1" s="10"/>
+      <c r="W1" s="10"/>
+      <c r="X1" s="10"/>
+      <c r="Y1" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="Z1" s="4"/>
-      <c r="AA1" s="4"/>
-      <c r="AB1" s="4"/>
-      <c r="AC1" s="4" t="s">
+      <c r="Z1" s="10"/>
+      <c r="AA1" s="10"/>
+      <c r="AB1" s="10"/>
+      <c r="AC1" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="AD1" s="4"/>
-      <c r="AE1" s="4"/>
+      <c r="AD1" s="10"/>
+      <c r="AE1" s="10"/>
     </row>
     <row r="2" spans="1:31" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
@@ -835,139 +835,139 @@
       </c>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="A3" s="8">
+      <c r="A3" s="4">
         <f>'Deployment Log'!A3</f>
         <v>0</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="4">
         <f>'Deployment Log'!N3</f>
         <v>0</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="4">
         <f>'Deployment Log'!O3</f>
         <v>0</v>
       </c>
-      <c r="D3" s="9">
+      <c r="D3" s="5">
         <f>'Deployment Log'!I3</f>
         <v>0</v>
       </c>
-      <c r="E3" s="9">
+      <c r="E3" s="5">
         <f>'Deployment Log'!J3</f>
         <v>0</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="5">
         <f>'Deployment Log'!K3</f>
         <v>0</v>
       </c>
-      <c r="G3" s="9">
+      <c r="G3" s="5">
         <f>'Recovery Log'!J3</f>
         <v>0</v>
       </c>
-      <c r="H3" s="9">
+      <c r="H3" s="5">
         <f>'Recovery Log'!K3</f>
         <v>0</v>
       </c>
-      <c r="I3" s="9">
-        <f>'Recovery Log'!L3</f>
-        <v>0</v>
-      </c>
-      <c r="J3" s="8">
+      <c r="I3" s="5">
+        <f>MIN('Recovery Log'!L3:M3)</f>
+        <v>0</v>
+      </c>
+      <c r="J3" s="4">
         <f>'Deployment Log'!B3</f>
         <v>0</v>
       </c>
-      <c r="K3" s="8">
+      <c r="K3" s="4">
         <f>'Deployment Log'!C3</f>
         <v>0</v>
       </c>
-      <c r="L3" s="8">
+      <c r="L3" s="4">
         <f>'Deployment Log'!D3</f>
         <v>0</v>
       </c>
-      <c r="M3" s="8">
+      <c r="M3" s="4">
         <f>'Deployment Log'!E3</f>
         <v>0</v>
       </c>
-      <c r="N3" s="8">
+      <c r="N3" s="4">
         <f>'Deployment Log'!F3</f>
         <v>0</v>
       </c>
-      <c r="O3" s="8">
+      <c r="O3" s="4">
         <f>'Deployment Log'!G3</f>
         <v>0</v>
       </c>
-      <c r="P3" s="10" t="str">
+      <c r="P3" s="6" t="str">
         <f>'Deployment Log'!H3</f>
         <v/>
       </c>
-      <c r="W3" s="12" t="str">
+      <c r="W3" s="8" t="str">
         <f>IF(ISBLANK(Q3),"",2*6370*ASIN(SQRT(SIN(RADIANS(Q3-M3)/2)*SIN(RADIANS(Q3-M3)/2) + COS(RADIANS(Q3))*COS(RADIANS(M3))*SIN(RADIANS(R3-N3)/2)*SIN(RADIANS(R3-N3)/2)))*1000)</f>
         <v/>
       </c>
-      <c r="X3" s="13" t="str">
+      <c r="X3" s="9" t="str">
         <f>IF(ISBLANK(Q3),"",MOD(DEGREES(ATAN2(COS(RADIANS(M3))*SIN(RADIANS(Q3)) - SIN(RADIANS(M3))*COS(RADIANS(Q3))*COS(RADIANS(R3-N3)),COS(RADIANS(Q3))*SIN(RADIANS(R3-N3)))) + 360, 360))</f>
         <v/>
       </c>
-      <c r="Y3" s="8">
+      <c r="Y3" s="4">
         <f>'Recovery Log'!N3</f>
         <v>0</v>
       </c>
-      <c r="Z3" s="8">
+      <c r="Z3" s="4">
         <f>'Recovery Log'!O3</f>
         <v>0</v>
       </c>
-      <c r="AA3" s="10" t="str">
+      <c r="AA3" s="6" t="str">
         <f>'Recovery Log'!P3</f>
         <v/>
       </c>
-      <c r="AB3" s="13" t="str">
+      <c r="AB3" s="9" t="str">
         <f>IF(ISBLANK(Q3),"",MOD(DEGREES(ATAN2(COS(RADIANS(Q3))*SIN(RADIANS(Y3)) - SIN(RADIANS(Q3))*COS(RADIANS(Y3))*COS(RADIANS(Z3-R3)),COS(RADIANS(Y3))*SIN(RADIANS(Z3-R3)))) + 360, 360))</f>
         <v/>
       </c>
-      <c r="AC3" s="8">
+      <c r="AC3" s="4">
         <f>'Recovery Log'!Q3</f>
         <v>0</v>
       </c>
-      <c r="AD3" s="8">
+      <c r="AD3" s="4">
         <f>'Recovery Log'!R3</f>
         <v>0</v>
       </c>
-      <c r="AE3" s="10" t="str">
+      <c r="AE3" s="6" t="str">
         <f>'Recovery Log'!S3</f>
         <v/>
       </c>
     </row>
     <row r="4" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P4" s="10"/>
+      <c r="P4" s="6"/>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P5" s="10"/>
+      <c r="P5" s="6"/>
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P6" s="10"/>
+      <c r="P6" s="6"/>
     </row>
     <row r="7" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P7" s="10"/>
+      <c r="P7" s="6"/>
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P8" s="10"/>
+      <c r="P8" s="6"/>
     </row>
     <row r="9" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P9" s="10"/>
+      <c r="P9" s="6"/>
     </row>
     <row r="10" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P10" s="10"/>
+      <c r="P10" s="6"/>
     </row>
     <row r="11" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P11" s="10"/>
+      <c r="P11" s="6"/>
     </row>
     <row r="12" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P12" s="10"/>
+      <c r="P12" s="6"/>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P13" s="10"/>
+      <c r="P13" s="6"/>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.25">
-      <c r="P14" s="10"/>
+      <c r="P14" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -1037,82 +1037,82 @@
   <dimension ref="A1:AA14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="8"/>
-    <col min="3" max="3" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="8"/>
-    <col min="6" max="6" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.140625" style="8" customWidth="1"/>
-    <col min="10" max="10" width="11.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.7109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.140625" style="8"/>
-    <col min="15" max="15" width="10" style="8" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="10" style="8" customWidth="1"/>
-    <col min="18" max="19" width="9.140625" style="8"/>
-    <col min="20" max="20" width="10.5703125" style="8" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9.140625" style="8"/>
-    <col min="22" max="22" width="20" style="8" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11" style="8" customWidth="1"/>
-    <col min="25" max="26" width="10.42578125" style="8" customWidth="1"/>
-    <col min="27" max="27" width="98.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="28" max="16384" width="9.140625" style="8"/>
+    <col min="1" max="1" width="13.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="4"/>
+    <col min="3" max="3" width="9.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="4"/>
+    <col min="6" max="6" width="9.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" style="4" customWidth="1"/>
+    <col min="10" max="10" width="11.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.140625" style="4"/>
+    <col min="15" max="15" width="10" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="10" style="4" customWidth="1"/>
+    <col min="18" max="19" width="9.140625" style="4"/>
+    <col min="20" max="20" width="10.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.140625" style="4"/>
+    <col min="22" max="22" width="20" style="4" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="11" style="4" customWidth="1"/>
+    <col min="25" max="26" width="10.42578125" style="4" customWidth="1"/>
+    <col min="27" max="27" width="98.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="28" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:27" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="5" t="s">
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5"/>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
-      <c r="N1" s="4" t="s">
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4" t="s">
+      <c r="O1" s="10"/>
+      <c r="P1" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="Q1" s="4"/>
-      <c r="R1" s="4" t="s">
+      <c r="Q1" s="10"/>
+      <c r="R1" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="S1" s="4"/>
-      <c r="T1" s="4" t="s">
+      <c r="S1" s="10"/>
+      <c r="T1" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="U1" s="4"/>
-      <c r="V1" s="4"/>
+      <c r="U1" s="10"/>
+      <c r="V1" s="10"/>
       <c r="W1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="X1" s="6" t="s">
+      <c r="X1" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="Y1" s="4" t="s">
+      <c r="Y1" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="Z1" s="4"/>
+      <c r="Z1" s="10"/>
       <c r="AA1" s="1" t="s">
         <v>13</v>
       </c>
@@ -1184,7 +1184,7 @@
       <c r="W2" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="X2" s="7"/>
+      <c r="X2" s="13"/>
       <c r="Y2" s="2" t="s">
         <v>54</v>
       </c>
@@ -1193,103 +1193,103 @@
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H3" s="12" t="str">
+      <c r="H3" s="8" t="str">
         <f>IF(OR(ISBLANK(B3),ISBLANK(E3)),"",2*6370*ASIN(SQRT(SIN(RADIANS(E3-B3)/2)*SIN(RADIANS(E3-B3)/2) + COS(RADIANS(E3))*COS(RADIANS(B3))*SIN(RADIANS(F3-C3)/2)*SIN(RADIANS(F3-C3)/2))))</f>
         <v/>
       </c>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="9"/>
-      <c r="M3" s="9"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H4" s="10"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H5" s="10"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="9"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H6" s="10"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="9"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H7" s="10"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H8" s="10"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="9"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H9" s="10"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="9"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H10" s="10"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="9"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H11" s="10"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
-      <c r="M11" s="9"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="5"/>
+      <c r="M11" s="5"/>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H12" s="10"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-      <c r="M12" s="9"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="5"/>
+      <c r="L12" s="5"/>
+      <c r="M12" s="5"/>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H13" s="10"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-      <c r="L13" s="9"/>
-      <c r="M13" s="9"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="H14" s="10"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-      <c r="L14" s="9"/>
-      <c r="M14" s="9"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -1325,66 +1325,66 @@
   <dimension ref="A1:X3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="8"/>
-    <col min="3" max="3" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="8" width="9.140625" style="8"/>
-    <col min="9" max="9" width="15.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.42578125" style="8" customWidth="1"/>
-    <col min="11" max="12" width="9.140625" style="8" customWidth="1"/>
-    <col min="13" max="13" width="17.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.140625" style="8" customWidth="1"/>
-    <col min="15" max="15" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.140625" style="8" customWidth="1"/>
-    <col min="18" max="18" width="9.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="16.7109375" style="8" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="9.140625" style="8"/>
-    <col min="22" max="22" width="11.42578125" style="8" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="20.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="100.5703125" style="8" customWidth="1"/>
-    <col min="25" max="16384" width="9.140625" style="8"/>
+    <col min="1" max="1" width="13.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" style="4"/>
+    <col min="3" max="3" width="9.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="8" width="9.140625" style="4"/>
+    <col min="9" max="9" width="15.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.42578125" style="4" customWidth="1"/>
+    <col min="11" max="12" width="9.140625" style="4" customWidth="1"/>
+    <col min="13" max="13" width="17.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.140625" style="4" customWidth="1"/>
+    <col min="15" max="15" width="9.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.140625" style="4" customWidth="1"/>
+    <col min="18" max="18" width="9.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="16.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="9.140625" style="4"/>
+    <col min="22" max="22" width="11.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="20.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="100.5703125" style="4" customWidth="1"/>
+    <col min="25" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4" t="s">
+      <c r="F1" s="10"/>
+      <c r="G1" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4" t="s">
+      <c r="H1" s="10"/>
+      <c r="I1" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4" t="s">
+      <c r="J1" s="10"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="10"/>
+      <c r="M1" s="10"/>
+      <c r="N1" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="4" t="s">
+      <c r="O1" s="10"/>
+      <c r="P1" s="10"/>
+      <c r="Q1" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="R1" s="4"/>
-      <c r="S1" s="4"/>
-      <c r="T1" s="4" t="s">
+      <c r="R1" s="10"/>
+      <c r="S1" s="10"/>
+      <c r="T1" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="U1" s="4"/>
+      <c r="U1" s="10"/>
       <c r="V1" s="1" t="s">
         <v>34</v>
       </c>
@@ -1461,31 +1461,31 @@
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A3" s="8">
+      <c r="A3" s="4">
         <f>'Deployment Log'!A3</f>
         <v>0</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="4">
         <f>'Deployment Log'!N3</f>
         <v>0</v>
       </c>
-      <c r="F3" s="8">
+      <c r="F3" s="4">
         <f>'Deployment Log'!O3</f>
         <v>0</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="4">
         <f>'Deployment Log'!R3</f>
         <v>0</v>
       </c>
-      <c r="H3" s="8">
+      <c r="H3" s="4">
         <f>'Deployment Log'!S3</f>
         <v>0</v>
       </c>
-      <c r="P3" s="12" t="str">
+      <c r="P3" s="8" t="str">
         <f>IF(ISBLANK(N3),"",2*6370*ASIN(SQRT(SIN(RADIANS(N3-B3)/2)*SIN(RADIANS(N3-B3)/2) + COS(RADIANS(N3))*COS(RADIANS(B3))*SIN(RADIANS(O3-C3)/2)*SIN(RADIANS(O3-C3)/2))))</f>
         <v/>
       </c>
-      <c r="S3" s="12" t="str">
+      <c r="S3" s="8" t="str">
         <f>IF(OR(ISBLANK(N3),ISBLANK(Q3)),"",2*6370*ASIN(SQRT(SIN(RADIANS(Q3-N3)/2)*SIN(RADIANS(Q3-N3)/2) + COS(RADIANS(Q3))*COS(RADIANS(N3))*SIN(RADIANS(R3-O3)/2)*SIN(RADIANS(R3-O3)/2))))</f>
         <v/>
       </c>

</xml_diff>